<commit_message>
feat(passion-lecture): JDT Thomas P
</commit_message>
<xml_diff>
--- a/Doc/X-Journal-de-Travail_PeltierThomas.xlsx
+++ b/Doc/X-Journal-de-Travail_PeltierThomas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv03xgo\Documents\GitHub\Passion-Lecture\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0371D1F-740D-4B36-A627-BF0EF8C564BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547C22FB-7B15-4B13-9A49-8B19BC4A70B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30765" yWindow="2715" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="55">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -197,6 +197,15 @@
   </si>
   <si>
     <t>J'ai aidez à régler le problème d'affichage sur la page détaille</t>
+  </si>
+  <si>
+    <t>Débrif du test avec la classe</t>
+  </si>
+  <si>
+    <t>J'ai continué le rapport</t>
+  </si>
+  <si>
+    <t>J'ai vérifier touts les points du cahier des charges et comparé avec ce que nous avons. J'ai du modifier certain point qui n'étais pas exactement ce que le cdc demandais notament dans le rapport</t>
   </si>
 </sst>
 </file>
@@ -1214,7 +1223,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>95</c:v>
+                  <c:v>210</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>365</c:v>
@@ -1223,7 +1232,7 @@
                   <c:v>110</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>645</c:v>
+                  <c:v>710</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -2069,16 +2078,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>7.8189300411522639E-2</c:v>
+                  <c:v>0.15053763440860216</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.30041152263374488</c:v>
+                  <c:v>0.26164874551971329</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.0534979423868317E-2</c:v>
+                  <c:v>7.8853046594982074E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.53086419753086422</c:v>
+                  <c:v>0.50896057347670254</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4313,7 +4322,7 @@
       <c r="B3" s="87"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>20 heures 15 minutes</v>
+        <v>23 heures 15 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4328,15 +4337,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>720</v>
+        <v>840</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>495</v>
+        <v>555</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1215</v>
+        <v>1395</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4944,39 +4953,67 @@
       <c r="G30" s="39"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="63" t="str">
+      <c r="A31" s="63">
         <f>IF(ISBLANK(B31),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B31))</f>
-        <v/>
-      </c>
-      <c r="B31" s="34"/>
+        <v>11</v>
+      </c>
+      <c r="B31" s="34">
+        <v>46092</v>
+      </c>
       <c r="C31" s="35"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="37"/>
-      <c r="F31" s="22"/>
+      <c r="D31" s="36">
+        <v>25</v>
+      </c>
+      <c r="E31" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" s="22" t="s">
+        <v>52</v>
+      </c>
       <c r="G31" s="40"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="62" t="str">
+      <c r="A32" s="62">
         <f>IF(ISBLANK(B32),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B32))</f>
-        <v/>
-      </c>
-      <c r="B32" s="30"/>
-      <c r="C32" s="31"/>
-      <c r="D32" s="32"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="23"/>
+        <v>11</v>
+      </c>
+      <c r="B32" s="30">
+        <v>46092</v>
+      </c>
+      <c r="C32" s="31">
+        <v>1</v>
+      </c>
+      <c r="D32" s="32">
+        <v>5</v>
+      </c>
+      <c r="E32" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="23" t="s">
+        <v>53</v>
+      </c>
       <c r="G32" s="39"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="63" t="str">
+      <c r="A33" s="63">
         <f>IF(ISBLANK(B33),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B33))</f>
-        <v/>
-      </c>
-      <c r="B33" s="34"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="36"/>
-      <c r="E33" s="37"/>
-      <c r="F33" s="22"/>
+        <v>11</v>
+      </c>
+      <c r="B33" s="34">
+        <v>46092</v>
+      </c>
+      <c r="C33" s="35">
+        <v>1</v>
+      </c>
+      <c r="D33" s="36">
+        <v>30</v>
+      </c>
+      <c r="E33" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" s="22" t="s">
+        <v>54</v>
+      </c>
       <c r="G33" s="40"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -11101,15 +11138,15 @@
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>95</v>
+        <v>210</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11117,11 +11154,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>1 h 35 min</v>
+        <v>3 h 30 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>7.8189300411522639E-2</v>
+        <v>0.15053763440860216</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11158,7 +11195,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.30041152263374488</v>
+        <v>0.26164874551971329</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11195,7 +11232,7 @@
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>9.0534979423868317E-2</v>
+        <v>7.8853046594982074E-2</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11212,15 +11249,15 @@
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>645</v>
+        <v>710</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11228,11 +11265,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>10 h 45 min</v>
+        <v>11 h 50 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.53086419753086422</v>
+        <v>0.50896057347670254</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11284,26 +11321,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>720</v>
+        <v>840</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>495</v>
+        <v>555</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1215</v>
+        <v>1395</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>30</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>20 h 15 min</v>
+        <v>23 h 15 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.22500000000000001</v>
+        <v>0.25833333333333336</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>30</v>
@@ -11342,15 +11379,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="b4a5ad45c54fa8cfccf4b5a6490850dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fe3b3ea8edd81a9012b97c6ddf640adc" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11539,6 +11567,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -11551,14 +11588,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B10C3F0-E765-401E-838F-B3E1E8C6407D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11577,6 +11606,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Doc(passion-lecture): update jdt Thomas P
</commit_message>
<xml_diff>
--- a/Doc/X-Journal-de-Travail_PeltierThomas.xlsx
+++ b/Doc/X-Journal-de-Travail_PeltierThomas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pv03xgo\Documents\GitHub\Passion-Lecture\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547C22FB-7B15-4B13-9A49-8B19BC4A70B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9699C9C7-66AB-4512-8C74-0500B4A5E99D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="57">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -206,6 +206,12 @@
   </si>
   <si>
     <t>J'ai vérifier touts les points du cahier des charges et comparé avec ce que nous avons. J'ai du modifier certain point qui n'étais pas exactement ce que le cdc demandais notament dans le rapport</t>
+  </si>
+  <si>
+    <t>J'ai préparer mon test</t>
+  </si>
+  <si>
+    <t>j'ai fais le test</t>
   </si>
 </sst>
 </file>
@@ -479,7 +485,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -680,6 +686,36 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1223,13 +1259,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>210</c:v>
+                  <c:v>255</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>365</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>110</c:v>
+                  <c:v>290</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>710</c:v>
@@ -2078,16 +2114,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.15053763440860216</c:v>
+                  <c:v>0.15740740740740741</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.26164874551971329</c:v>
+                  <c:v>0.22530864197530864</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.8853046594982074E-2</c:v>
+                  <c:v>0.17901234567901234</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.50896057347670254</c:v>
+                  <c:v>0.43827160493827161</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4322,7 +4358,7 @@
       <c r="B3" s="87"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>23 heures 15 minutes</v>
+        <v>27 heures 0 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4337,15 +4373,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>840</v>
+        <v>1020</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>555</v>
+        <v>600</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1395</v>
+        <v>1620</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4954,90 +4990,108 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="63">
-        <f>IF(ISBLANK(B31),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B31))</f>
+        <f>IF(ISBLANK(B33),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B33))</f>
         <v>11</v>
       </c>
-      <c r="B31" s="34">
-        <v>46092</v>
-      </c>
-      <c r="C31" s="35"/>
-      <c r="D31" s="36">
-        <v>25</v>
-      </c>
-      <c r="E31" s="37" t="s">
+      <c r="B31" s="88">
+        <v>46091</v>
+      </c>
+      <c r="C31" s="90"/>
+      <c r="D31" s="92">
+        <v>45</v>
+      </c>
+      <c r="E31" s="94" t="s">
         <v>17</v>
       </c>
-      <c r="F31" s="22" t="s">
-        <v>52</v>
+      <c r="F31" s="96" t="s">
+        <v>55</v>
       </c>
       <c r="G31" s="40"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="62">
-        <f>IF(ISBLANK(B32),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B32))</f>
+        <f>IF(ISBLANK(B34),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B34))</f>
         <v>11</v>
       </c>
-      <c r="B32" s="30">
-        <v>46092</v>
-      </c>
-      <c r="C32" s="31">
-        <v>1</v>
-      </c>
-      <c r="D32" s="32">
-        <v>5</v>
-      </c>
-      <c r="E32" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="F32" s="23" t="s">
-        <v>53</v>
+      <c r="B32" s="88">
+        <v>46091</v>
+      </c>
+      <c r="C32" s="90">
+        <v>3</v>
+      </c>
+      <c r="D32" s="92">
+        <v>0</v>
+      </c>
+      <c r="E32" s="94" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="96" t="s">
+        <v>56</v>
       </c>
       <c r="G32" s="39"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="63">
-        <f>IF(ISBLANK(B33),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B33))</f>
+        <f>IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
         <v>11</v>
       </c>
-      <c r="B33" s="34">
+      <c r="B33" s="89">
         <v>46092</v>
       </c>
-      <c r="C33" s="35">
+      <c r="C33" s="91"/>
+      <c r="D33" s="93">
+        <v>25</v>
+      </c>
+      <c r="E33" s="95" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" s="96" t="s">
+        <v>52</v>
+      </c>
+      <c r="G33" s="40"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="62" t="e">
+        <f>IF(ISBLANK(#REF!),"",_xlfn.ISOWEEKNUM('Journal de travail'!#REF!))</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B34" s="88">
+        <v>46092</v>
+      </c>
+      <c r="C34" s="90">
         <v>1</v>
       </c>
-      <c r="D33" s="36">
+      <c r="D34" s="92">
+        <v>5</v>
+      </c>
+      <c r="E34" s="94" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" s="96" t="s">
+        <v>53</v>
+      </c>
+      <c r="G34" s="39"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="63" t="e">
+        <f>IF(ISBLANK(#REF!),"",_xlfn.ISOWEEKNUM('Journal de travail'!#REF!))</f>
+        <v>#REF!</v>
+      </c>
+      <c r="B35" s="34">
+        <v>46092</v>
+      </c>
+      <c r="C35" s="35">
+        <v>1</v>
+      </c>
+      <c r="D35" s="36">
         <v>30</v>
       </c>
-      <c r="E33" s="37" t="s">
+      <c r="E35" s="37" t="s">
         <v>17</v>
       </c>
-      <c r="F33" s="22" t="s">
+      <c r="F35" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="G33" s="40"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="62" t="str">
-        <f>IF(ISBLANK(B34),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B34))</f>
-        <v/>
-      </c>
-      <c r="B34" s="30"/>
-      <c r="C34" s="31"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="22"/>
-      <c r="G34" s="39"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="63" t="str">
-        <f>IF(ISBLANK(B35),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B35))</f>
-        <v/>
-      </c>
-      <c r="B35" s="34"/>
-      <c r="C35" s="35"/>
-      <c r="D35" s="36"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="23"/>
       <c r="G35" s="40"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -11012,7 +11066,7 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E7:E532">
+  <conditionalFormatting sqref="E7:E30 E33:E532">
     <cfRule type="expression" dxfId="8" priority="1">
       <formula>$E7="Absent"</formula>
     </cfRule>
@@ -11042,13 +11096,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C532" xr:uid="{9D52E29F-610D-40B2-B3CC-F94A741DD978}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C30 C33:C532" xr:uid="{9D52E29F-610D-40B2-B3CC-F94A741DD978}">
       <formula1>$N$7:$N$15</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D532" xr:uid="{46510F84-8BCC-4BD6-9A19-9F03ACD74D05}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D30 D33:D532" xr:uid="{46510F84-8BCC-4BD6-9A19-9F03ACD74D05}">
       <formula1>$O$7:$O$19</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E532" xr:uid="{EBCA439E-C5F1-BC4C-88EE-2BB045537E3E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E30 E33:E532" xr:uid="{EBCA439E-C5F1-BC4C-88EE-2BB045537E3E}">
       <formula1>$M$7:$M$12</formula1>
     </dataValidation>
   </dataValidations>
@@ -11142,11 +11196,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>150</v>
+        <v>195</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>210</v>
+        <v>255</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11154,11 +11208,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>3 h 30 min</v>
+        <v>4 h 15 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.15053763440860216</v>
+        <v>0.15740740740740741</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11195,7 +11249,7 @@
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.26164874551971329</v>
+        <v>0.22530864197530864</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11212,7 +11266,7 @@
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E8,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>60</v>
+        <v>240</v>
       </c>
       <c r="B8">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E8,'Journal de travail'!$D$7:$D$532)</f>
@@ -11220,7 +11274,7 @@
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
-        <v>110</v>
+        <v>290</v>
       </c>
       <c r="E8" s="76" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11228,11 +11282,11 @@
       </c>
       <c r="F8" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>1 h 50 min</v>
+        <v>4 h 50 min</v>
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>7.8853046594982074E-2</v>
+        <v>0.17901234567901234</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11269,7 +11323,7 @@
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.50896057347670254</v>
+        <v>0.43827160493827161</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11321,26 +11375,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>840</v>
+        <v>1020</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>555</v>
+        <v>600</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1395</v>
+        <v>1620</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>30</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>23 h 15 min</v>
+        <v>27 h 00 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.25833333333333336</v>
+        <v>0.3</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>30</v>
@@ -11379,6 +11433,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="b4a5ad45c54fa8cfccf4b5a6490850dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fe3b3ea8edd81a9012b97c6ddf640adc" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11567,15 +11630,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -11588,6 +11642,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B10C3F0-E765-401E-838F-B3E1E8C6407D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11606,14 +11668,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>

</xml_diff>